<commit_message>
Weekly Digital Demand Pulse
</commit_message>
<xml_diff>
--- a/excel/Digital-Demand-Pulse.xlsx
+++ b/excel/Digital-Demand-Pulse.xlsx
@@ -480,19 +480,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>153160</v>
+        <v>152556</v>
       </c>
       <c r="E2" t="n">
-        <v>201737</v>
+        <v>201002</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.2407937066576781</v>
+        <v>-0.2410224773882846</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5737361023704636</v>
+        <v>0.5740259251594454</v>
       </c>
       <c r="H2" t="n">
-        <v>0.5083085776773274</v>
+        <v>0.5088542286378285</v>
       </c>
     </row>
     <row r="3">
@@ -512,19 +512,19 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>52239</v>
+        <v>52033</v>
       </c>
       <c r="E3" t="n">
-        <v>98957</v>
+        <v>98287</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.4721040451913457</v>
+        <v>-0.4706014020165434</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1956868650543918</v>
+        <v>0.1957857505691118</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2493379594284404</v>
+        <v>0.2488221787351681</v>
       </c>
     </row>
     <row r="4">
@@ -544,19 +544,19 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>23984</v>
+        <v>23845</v>
       </c>
       <c r="E4" t="n">
-        <v>37807</v>
+        <v>37592</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.3656201232575979</v>
+        <v>-0.3656895084060439</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0898438670622434</v>
+        <v>0.08972212292815081</v>
       </c>
       <c r="H4" t="n">
-        <v>0.09526077217489462</v>
+        <v>0.09516745188084322</v>
       </c>
     </row>
     <row r="5">
@@ -576,19 +576,19 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>23325</v>
+        <v>23205</v>
       </c>
       <c r="E5" t="n">
-        <v>37784</v>
+        <v>37612</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.3826752064365869</v>
+        <v>-0.383042645964054</v>
       </c>
       <c r="G5" t="n">
-        <v>0.08737525847343343</v>
+        <v>0.0873139803962147</v>
       </c>
       <c r="H5" t="n">
-        <v>0.09520282000307398</v>
+        <v>0.09521808363860064</v>
       </c>
     </row>
     <row r="6">
@@ -608,19 +608,19 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>14244</v>
+        <v>14126</v>
       </c>
       <c r="E6" t="n">
-        <v>20594</v>
+        <v>20516</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.3083422356026027</v>
+        <v>-0.311464223045428</v>
       </c>
       <c r="G6" t="n">
-        <v>0.05335790703946777</v>
+        <v>0.05315222094707731</v>
       </c>
       <c r="H6" t="n">
-        <v>0.05188987071626365</v>
+        <v>0.05193805710755958</v>
       </c>
     </row>
     <row r="7">
@@ -640,19 +640,19 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>57640</v>
+        <v>57485</v>
       </c>
       <c r="E7" t="n">
-        <v>109595</v>
+        <v>108830</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.47406359779187</v>
+        <v>-0.4717908664890196</v>
       </c>
       <c r="G7" t="n">
-        <v>0.03468192093556949</v>
+        <v>0.0347771533733869</v>
       </c>
       <c r="H7" t="n">
-        <v>0.02652654397096276</v>
+        <v>0.02659894928895531</v>
       </c>
     </row>
     <row r="8">
@@ -672,19 +672,19 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>23502</v>
+        <v>23352</v>
       </c>
       <c r="E8" t="n">
-        <v>62416</v>
+        <v>61689</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.623461932837734</v>
+        <v>-0.6214560132276419</v>
       </c>
       <c r="G8" t="n">
-        <v>0.01414112605530455</v>
+        <v>0.01412744343003098</v>
       </c>
       <c r="H8" t="n">
-        <v>0.01510726555492141</v>
+        <v>0.01507730021764554</v>
       </c>
     </row>
     <row r="9">
@@ -704,19 +704,19 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>150322</v>
+        <v>149426</v>
       </c>
       <c r="E9" t="n">
-        <v>279692</v>
+        <v>278838</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.4625445132502896</v>
+        <v>-0.4641117781650994</v>
       </c>
       <c r="G9" t="n">
-        <v>0.09044857249959536</v>
+        <v>0.0903994245450415</v>
       </c>
       <c r="H9" t="n">
-        <v>0.06769708596493011</v>
+        <v>0.06815030618242876</v>
       </c>
     </row>
     <row r="10">
@@ -736,19 +736,19 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>234013</v>
+        <v>234026</v>
       </c>
       <c r="E10" t="n">
-        <v>348454</v>
+        <v>344054</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.3284249857943947</v>
+        <v>-0.319798636260587</v>
       </c>
       <c r="G10" t="n">
-        <v>0.140805349824695</v>
+        <v>0.1415805531070757</v>
       </c>
       <c r="H10" t="n">
-        <v>0.08434034721344821</v>
+        <v>0.0840896342797228</v>
       </c>
     </row>
     <row r="11">
@@ -768,19 +768,19 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>685634</v>
+        <v>681352</v>
       </c>
       <c r="E11" t="n">
-        <v>1958001</v>
+        <v>1935785</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.6498295966140977</v>
+        <v>-0.64802289510457</v>
       </c>
       <c r="G11" t="n">
-        <v>0.4125451800613853</v>
+        <v>0.4122028878014076</v>
       </c>
       <c r="H11" t="n">
-        <v>0.4739176022782887</v>
+        <v>0.4731218142912833</v>
       </c>
     </row>
     <row r="12">
@@ -800,19 +800,19 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>510850</v>
+        <v>507312</v>
       </c>
       <c r="E12" t="n">
-        <v>1373364</v>
+        <v>1362319</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.6280301507830408</v>
+        <v>-0.6276114478327028</v>
       </c>
       <c r="G12" t="n">
-        <v>0.3073778506234502</v>
+        <v>0.3069125377430574</v>
       </c>
       <c r="H12" t="n">
-        <v>0.3324111550174488</v>
+        <v>0.3329619957399643</v>
       </c>
     </row>
     <row r="13">
@@ -832,19 +832,19 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>131127</v>
+        <v>130590</v>
       </c>
       <c r="E13" t="n">
-        <v>240158</v>
+        <v>237111</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.4539969520065956</v>
+        <v>-0.4492452901805484</v>
       </c>
       <c r="G13" t="n">
-        <v>0.6538565102920058</v>
+        <v>0.6546389685388302</v>
       </c>
       <c r="H13" t="n">
-        <v>0.5822887318821253</v>
+        <v>0.5811515629825345</v>
       </c>
     </row>
     <row r="14">
@@ -864,19 +864,19 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>44245</v>
+        <v>43921</v>
       </c>
       <c r="E14" t="n">
-        <v>117205</v>
+        <v>116339</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.6224990401433386</v>
+        <v>-0.6224739769122993</v>
       </c>
       <c r="G14" t="n">
-        <v>0.2206249002712622</v>
+        <v>0.2201730464598665</v>
       </c>
       <c r="H14" t="n">
-        <v>0.2841760458541647</v>
+        <v>0.2851432100823035</v>
       </c>
     </row>
     <row r="15">
@@ -896,19 +896,19 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>25172</v>
+        <v>24973</v>
       </c>
       <c r="E15" t="n">
-        <v>55075</v>
+        <v>54552</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.5429505220154335</v>
+        <v>-0.5422166006745857</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1255185894367321</v>
+        <v>0.1251879850013034</v>
       </c>
       <c r="H15" t="n">
-        <v>0.13353522226371</v>
+        <v>0.1337052269351621</v>
       </c>
     </row>
     <row r="16">
@@ -928,19 +928,19 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>13131</v>
+        <v>13050</v>
       </c>
       <c r="E16" t="n">
-        <v>19955</v>
+        <v>19921</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.3419694312202456</v>
+        <v>-0.3449124039957834</v>
       </c>
       <c r="G16" t="n">
-        <v>0.4403272861406392</v>
+        <v>0.4401645979492714</v>
       </c>
       <c r="H16" t="n">
-        <v>0.4315994376554558</v>
+        <v>0.4331217115275905</v>
       </c>
     </row>
     <row r="17">
@@ -960,19 +960,19 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>8318</v>
+        <v>8279</v>
       </c>
       <c r="E17" t="n">
-        <v>12613</v>
+        <v>12493</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.3405216839768492</v>
+        <v>-0.3373088929800688</v>
       </c>
       <c r="G17" t="n">
-        <v>0.2789309546963549</v>
+        <v>0.2792431192660551</v>
       </c>
       <c r="H17" t="n">
-        <v>0.272801989834541</v>
+        <v>0.2716223855285472</v>
       </c>
     </row>
     <row r="18">
@@ -992,19 +992,19 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>8372</v>
+        <v>8319</v>
       </c>
       <c r="E18" t="n">
-        <v>13667</v>
+        <v>13580</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.3874295748884173</v>
+        <v>-0.3874079528718704</v>
       </c>
       <c r="G18" t="n">
-        <v>0.2807417591630059</v>
+        <v>0.2805922827846735</v>
       </c>
       <c r="H18" t="n">
-        <v>0.2955985725100033</v>
+        <v>0.2952559029438622</v>
       </c>
     </row>
   </sheetData>
@@ -1060,76 +1060,76 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5754</v>
+        <v>5916</v>
       </c>
       <c r="D2" t="n">
-        <v>4606.8</v>
+        <v>4591.8</v>
       </c>
       <c r="E2" t="n">
-        <v>0.249</v>
+        <v>0.2884</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Atezolizumab</t>
+          <t>Cemiplimab</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tecentriq (atezolizumab)</t>
+          <t>Libtayo (cemiplimab)</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>466</v>
+        <v>179</v>
       </c>
       <c r="D3" t="n">
-        <v>373.8</v>
+        <v>242.2</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2468</v>
+        <v>-0.2611</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Rotavirus vaccine</t>
+          <t>Selexipag</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Rotavirus vaccine (RotaTeq, Rotarix)</t>
+          <t>Uptravi (selexipag)</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>205</v>
+        <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>267.2</v>
+        <v>131.5</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.2329</v>
+        <v>-0.2395</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cemiplimab</t>
+          <t>Rotavirus vaccine</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Libtayo (cemiplimab)</t>
+          <t>Rotavirus vaccine (RotaTeq, Rotarix)</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>188</v>
+        <v>206</v>
       </c>
       <c r="D5" t="n">
-        <v>243.8</v>
+        <v>263.2</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.2287</v>
+        <v>-0.2175</v>
       </c>
     </row>
     <row r="6">
@@ -1144,139 +1144,139 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2088</v>
+        <v>2038</v>
       </c>
       <c r="D6" t="n">
-        <v>2649.2</v>
+        <v>2522.2</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.2119</v>
+        <v>-0.192</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Nivolumab</t>
+          <t>Linagliptin</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Opdivo (nivolumab)</t>
+          <t>Trajenta (linagliptin)</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>716</v>
+        <v>343</v>
       </c>
       <c r="D7" t="n">
-        <v>884.5</v>
+        <v>413.5</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.1905</v>
+        <v>-0.1705</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Linagliptin</t>
+          <t>Tirzepatide</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Trajenta (linagliptin)</t>
+          <t>Mounjaro/Zepbound (tirzepatide)</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>354</v>
+        <v>6802</v>
       </c>
       <c r="D8" t="n">
-        <v>432.5</v>
+        <v>7980.2</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.1815</v>
+        <v>-0.1476</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Empagliflozin</t>
+          <t>Macitentan</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Jardiance (empagliflozin)</t>
+          <t>Opsumit (macitentan)</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1435</v>
+        <v>132</v>
       </c>
       <c r="D9" t="n">
-        <v>1736.2</v>
+        <v>154.5</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.1735</v>
+        <v>-0.1456</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tirzepatide</t>
+          <t>Semaglutide</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Mounjaro/Zepbound (tirzepatide)</t>
+          <t>Ozempic/Wegovy (semaglutide)</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6820</v>
+        <v>7758</v>
       </c>
       <c r="D10" t="n">
-        <v>8136</v>
+        <v>9068.799999999999</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.1618</v>
+        <v>-0.1445</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Semaglutide</t>
+          <t>Pneumococcal vaccine</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Ozempic/Wegovy (semaglutide)</t>
+          <t>Pneumococcal vaccine (Capvaxive, Vaxneuvance, Prevnar)</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>7860</v>
+        <v>1043</v>
       </c>
       <c r="D11" t="n">
-        <v>9197</v>
+        <v>914.5</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.1454</v>
+        <v>0.1405</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Selexipag</t>
+          <t>Pulmonary hypertension</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Uptravi (selexipag)</t>
+          <t>Pulmonary hypertension</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>115</v>
+        <v>1662</v>
       </c>
       <c r="D12" t="n">
-        <v>134.2</v>
+        <v>1904.8</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.1434</v>
+        <v>-0.1274</v>
       </c>
     </row>
     <row r="13">
@@ -1291,223 +1291,223 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="D13" t="n">
-        <v>409</v>
+        <v>402</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.132</v>
+        <v>-0.1219</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sitagliptin</t>
+          <t>Empagliflozin</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Januvia (sitagliptin)</t>
+          <t>Jardiance (empagliflozin)</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1137</v>
+        <v>1497</v>
       </c>
       <c r="D14" t="n">
-        <v>1267</v>
+        <v>1695.8</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.1026</v>
+        <v>-0.1172</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Pulmonary hypertension</t>
+          <t>Nivolumab</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Pulmonary hypertension</t>
+          <t>Opdivo (nivolumab)</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1709</v>
+        <v>775</v>
       </c>
       <c r="D15" t="n">
-        <v>1899.8</v>
+        <v>868.8</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.1004</v>
+        <v>-0.1079</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Cervical cancer</t>
+          <t>Sitagliptin</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cervical cancer</t>
+          <t>Januvia (sitagliptin)</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3163</v>
+        <v>1124</v>
       </c>
       <c r="D16" t="n">
-        <v>2884</v>
+        <v>1248.2</v>
       </c>
       <c r="E16" t="n">
-        <v>0.09669999999999999</v>
+        <v>-0.09950000000000001</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Pneumococcal vaccine</t>
+          <t>Dapagliflozin</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Pneumococcal vaccine (Capvaxive, Vaxneuvance, Prevnar)</t>
+          <t>Farxiga (dapagliflozin)</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>979</v>
+        <v>4921</v>
       </c>
       <c r="D17" t="n">
-        <v>922</v>
+        <v>5193.5</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0618</v>
+        <v>-0.0525</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Macitentan</t>
+          <t>Type 2 diabetes</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Opsumit (macitentan)</t>
+          <t>Type 2 diabetes</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>144</v>
+        <v>3455</v>
       </c>
       <c r="D18" t="n">
-        <v>153.2</v>
+        <v>3644.8</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.0604</v>
+        <v>-0.0521</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Type 2 diabetes</t>
+          <t>Atezolizumab</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Type 2 diabetes</t>
+          <t>Tecentriq (atezolizumab)</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3498</v>
+        <v>401</v>
       </c>
       <c r="D19" t="n">
-        <v>3704.2</v>
+        <v>383.8</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.0557</v>
+        <v>0.045</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Dapagliflozin</t>
+          <t>HPV vaccine</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Farxiga (dapagliflozin)</t>
+          <t>HPV vaccine (Gardasil)</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>5053</v>
+        <v>1556</v>
       </c>
       <c r="D20" t="n">
-        <v>5149.5</v>
+        <v>1612.5</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.0187</v>
+        <v>-0.035</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Melanoma</t>
+          <t>Sotatercept</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Melanoma</t>
+          <t>Winrevair (sotatercept)</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>7282</v>
+        <v>167</v>
       </c>
       <c r="D21" t="n">
-        <v>7390.2</v>
+        <v>163.2</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.0146</v>
+        <v>0.023</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>HPV vaccine</t>
+          <t>Cervical cancer</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>HPV vaccine (Gardasil)</t>
+          <t>Cervical cancer</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1599</v>
+        <v>2989</v>
       </c>
       <c r="D22" t="n">
-        <v>1620.5</v>
+        <v>2926.8</v>
       </c>
       <c r="E22" t="n">
-        <v>-0.0133</v>
+        <v>0.0213</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sotatercept</t>
+          <t>Melanoma</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Winrevair (sotatercept)</t>
+          <t>Melanoma</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>168</v>
+        <v>7211</v>
       </c>
       <c r="D23" t="n">
-        <v>167.8</v>
+        <v>7366.2</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0015</v>
+        <v>-0.0211</v>
       </c>
     </row>
   </sheetData>
@@ -2915,13 +2915,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>738</v>
+        <v>732</v>
       </c>
       <c r="F2" t="n">
-        <v>153160</v>
+        <v>152556</v>
       </c>
       <c r="G2" t="n">
-        <v>0.004818490467484983</v>
+        <v>0.00479823802406985</v>
       </c>
     </row>
     <row r="3">
@@ -2946,13 +2946,13 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="F3" t="n">
-        <v>52239</v>
+        <v>52033</v>
       </c>
       <c r="G3" t="n">
-        <v>0.004441126361530657</v>
+        <v>0.004381834604962236</v>
       </c>
     </row>
     <row r="4">
@@ -2977,13 +2977,13 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F4" t="n">
-        <v>23984</v>
+        <v>23845</v>
       </c>
       <c r="G4" t="n">
-        <v>0.006254169446297531</v>
+        <v>0.006248689452715454</v>
       </c>
     </row>
     <row r="5">
@@ -3008,13 +3008,13 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F5" t="n">
-        <v>23325</v>
+        <v>23205</v>
       </c>
       <c r="G5" t="n">
-        <v>0.004844587352625938</v>
+        <v>0.004783451842275372</v>
       </c>
     </row>
     <row r="6">
@@ -3042,10 +3042,10 @@
         <v>55</v>
       </c>
       <c r="F6" t="n">
-        <v>14244</v>
+        <v>14126</v>
       </c>
       <c r="G6" t="n">
-        <v>0.003861274922774501</v>
+        <v>0.003893529661616876</v>
       </c>
     </row>
     <row r="7">
@@ -3070,13 +3070,13 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="F7" t="n">
-        <v>57640</v>
+        <v>57485</v>
       </c>
       <c r="G7" t="n">
-        <v>0.008414295628036085</v>
+        <v>0.00841958771853527</v>
       </c>
     </row>
     <row r="8">
@@ -3101,13 +3101,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>601</v>
+        <v>596</v>
       </c>
       <c r="F8" t="n">
-        <v>23502</v>
+        <v>23352</v>
       </c>
       <c r="G8" t="n">
-        <v>0.02557229171985363</v>
+        <v>0.02552243919150394</v>
       </c>
     </row>
     <row r="9">
@@ -3132,13 +3132,13 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>2834</v>
+        <v>2769</v>
       </c>
       <c r="F9" t="n">
-        <v>150322</v>
+        <v>149426</v>
       </c>
       <c r="G9" t="n">
-        <v>0.01885286252178656</v>
+        <v>0.01853091162180611</v>
       </c>
     </row>
     <row r="10">
@@ -3163,13 +3163,13 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1447</v>
+        <v>1436</v>
       </c>
       <c r="F10" t="n">
-        <v>234013</v>
+        <v>234026</v>
       </c>
       <c r="G10" t="n">
-        <v>0.006183417160585096</v>
+        <v>0.006136070351157564</v>
       </c>
     </row>
     <row r="11">
@@ -3194,13 +3194,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>3119</v>
+        <v>3079</v>
       </c>
       <c r="F11" t="n">
-        <v>685634</v>
+        <v>681352</v>
       </c>
       <c r="G11" t="n">
-        <v>0.004549074287447822</v>
+        <v>0.00451895642780824</v>
       </c>
     </row>
     <row r="12">
@@ -3225,13 +3225,13 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>3730</v>
+        <v>3699</v>
       </c>
       <c r="F12" t="n">
-        <v>510850</v>
+        <v>507312</v>
       </c>
       <c r="G12" t="n">
-        <v>0.007301556229813056</v>
+        <v>0.007291370990632983</v>
       </c>
     </row>
     <row r="13">
@@ -3256,13 +3256,13 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2552</v>
+        <v>2516</v>
       </c>
       <c r="F13" t="n">
-        <v>131127</v>
+        <v>130590</v>
       </c>
       <c r="G13" t="n">
-        <v>0.01946204824330611</v>
+        <v>0.01926640630982464</v>
       </c>
     </row>
     <row r="14">
@@ -3287,13 +3287,13 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="F14" t="n">
-        <v>44245</v>
+        <v>43921</v>
       </c>
       <c r="G14" t="n">
-        <v>0.01796813199231552</v>
+        <v>0.0181462170715603</v>
       </c>
     </row>
     <row r="15">
@@ -3318,13 +3318,13 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>502</v>
+        <v>494</v>
       </c>
       <c r="F15" t="n">
-        <v>25172</v>
+        <v>24973</v>
       </c>
       <c r="G15" t="n">
-        <v>0.01994279358016844</v>
+        <v>0.01978136387298282</v>
       </c>
     </row>
     <row r="16">
@@ -3346,7 +3346,7 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
-        <v>13131</v>
+        <v>13050</v>
       </c>
       <c r="G16" t="inlineStr"/>
     </row>
@@ -3372,13 +3372,13 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F17" t="n">
-        <v>8318</v>
+        <v>8279</v>
       </c>
       <c r="G17" t="n">
-        <v>0.03402260158691994</v>
+        <v>0.03406208479284938</v>
       </c>
     </row>
     <row r="18">
@@ -3406,10 +3406,10 @@
         <v>100</v>
       </c>
       <c r="F18" t="n">
-        <v>8372</v>
+        <v>8319</v>
       </c>
       <c r="G18" t="n">
-        <v>0.01194457716196847</v>
+        <v>0.01202067556196658</v>
       </c>
     </row>
     <row r="19">
@@ -3434,13 +3434,13 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>15684</v>
+        <v>15648</v>
       </c>
       <c r="F19" t="n">
-        <v>314829</v>
+        <v>313786</v>
       </c>
       <c r="G19" t="n">
-        <v>0.04981751998704059</v>
+        <v>0.04986838163589197</v>
       </c>
     </row>
     <row r="20">
@@ -3465,13 +3465,13 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>5041</v>
+        <v>5039</v>
       </c>
       <c r="F20" t="n">
-        <v>434794</v>
+        <v>433637</v>
       </c>
       <c r="G20" t="n">
-        <v>0.01159399623729858</v>
+        <v>0.01162031837689127</v>
       </c>
     </row>
     <row r="21">
@@ -3496,13 +3496,13 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>3586</v>
+        <v>3564</v>
       </c>
       <c r="F21" t="n">
-        <v>233529</v>
+        <v>232504</v>
       </c>
       <c r="G21" t="n">
-        <v>0.01535569458182924</v>
+        <v>0.01532876853731549</v>
       </c>
     </row>
     <row r="22">
@@ -3527,13 +3527,13 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>2954</v>
+        <v>2901</v>
       </c>
       <c r="F22" t="n">
-        <v>153253</v>
+        <v>153295</v>
       </c>
       <c r="G22" t="n">
-        <v>0.01927531598076384</v>
+        <v>0.01892429629146417</v>
       </c>
     </row>
     <row r="23">
@@ -3558,13 +3558,13 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>1406</v>
+        <v>1382</v>
       </c>
       <c r="F23" t="n">
-        <v>125035</v>
+        <v>124715</v>
       </c>
       <c r="G23" t="n">
-        <v>0.01124485144159635</v>
+        <v>0.01108126528484946</v>
       </c>
     </row>
   </sheetData>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5,349 of 146,479 series-days, mostly small Arabic articles</t>
+          <t>5,358 of 146,608 series-days, mostly small Arabic articles</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -3707,7 +3707,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>146,479 rows</t>
+          <t>146,608 rows</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">

</xml_diff>